<commit_message>
Ajoute le contact issu du magazine municipal de Saint-Pierre (974)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SnYRwvFTou9edwhoWU27Hk
</commit_message>
<xml_diff>
--- a/associations_974_la_reunion.xlsx
+++ b/associations_974_la_reunion.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="communes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'contacts'!$A$1:$H$955</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'contacts'!$A$1:$H$956</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H955"/>
+  <dimension ref="A1:H956"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -35662,28 +35662,32 @@
     <row r="857">
       <c r="A857" t="inlineStr">
         <is>
-          <t>Association Domin Galizé</t>
+          <t>Lalanbik</t>
         </is>
       </c>
       <c r="B857" t="inlineStr">
         <is>
-          <t>Trois-Bassins</t>
+          <t>Saint-Pierre</t>
         </is>
       </c>
       <c r="C857" t="inlineStr">
         <is>
-          <t>domingalize@gmail.com</t>
-        </is>
-      </c>
-      <c r="D857" t="inlineStr"/>
+          <t>info@lalanbik.re</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>06 92 37 89 34</t>
+        </is>
+      </c>
       <c r="E857" t="inlineStr">
         <is>
-          <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
+          <t>https://www.saintpierre.re/sites/default/files/2023-04/VDS%20123%20V_4.pdf</t>
         </is>
       </c>
       <c r="F857" t="inlineStr">
         <is>
-          <t>2023-11-21 (PDF annuaire des associations de Trois Bassins, MAJ 21/11/2023, docs.trois-bassins.re; site actif 2026)</t>
+          <t>Mars 2023 - magazine municipal La VDS n°123 (PDF publié sur saintpierre.re, avril 2023) : programmation danse du Théâtre de Pierrefonds, ligne 'Réservation : Info@lalanbik.re ou 06 92 37 89 34' ; p.12 cite 'l'association Lalanbik' (convention avec la commune)</t>
         </is>
       </c>
       <c r="G857" t="inlineStr">
@@ -35700,7 +35704,7 @@
     <row r="858">
       <c r="A858" t="inlineStr">
         <is>
-          <t>Association Lo Ker Rényoné</t>
+          <t>Association Domin Galizé</t>
         </is>
       </c>
       <c r="B858" t="inlineStr">
@@ -35710,14 +35714,10 @@
       </c>
       <c r="C858" t="inlineStr">
         <is>
-          <t>laurence.bhiki@gmail.com</t>
-        </is>
-      </c>
-      <c r="D858" t="inlineStr">
-        <is>
-          <t>0692 94 14 59</t>
-        </is>
-      </c>
+          <t>domingalize@gmail.com</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr"/>
       <c r="E858" t="inlineStr">
         <is>
           <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
@@ -35742,7 +35742,7 @@
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t>Femmes Actives Manuelles</t>
+          <t>Association Lo Ker Rényoné</t>
         </is>
       </c>
       <c r="B859" t="inlineStr">
@@ -35752,12 +35752,12 @@
       </c>
       <c r="C859" t="inlineStr">
         <is>
-          <t>chamand.mpierre@gmail.com</t>
+          <t>laurence.bhiki@gmail.com</t>
         </is>
       </c>
       <c r="D859" t="inlineStr">
         <is>
-          <t>0692 56 35 29</t>
+          <t>0692 94 14 59</t>
         </is>
       </c>
       <c r="E859" t="inlineStr">
@@ -35784,7 +35784,7 @@
     <row r="860">
       <c r="A860" t="inlineStr">
         <is>
-          <t>Ile en alu</t>
+          <t>Femmes Actives Manuelles</t>
         </is>
       </c>
       <c r="B860" t="inlineStr">
@@ -35794,12 +35794,12 @@
       </c>
       <c r="C860" t="inlineStr">
         <is>
-          <t>pougary.davila@orange.fr</t>
+          <t>chamand.mpierre@gmail.com</t>
         </is>
       </c>
       <c r="D860" t="inlineStr">
         <is>
-          <t>0692 01 24 79</t>
+          <t>0692 56 35 29</t>
         </is>
       </c>
       <c r="E860" t="inlineStr">
@@ -35826,7 +35826,7 @@
     <row r="861">
       <c r="A861" t="inlineStr">
         <is>
-          <t>Mathias Maloya</t>
+          <t>Ile en alu</t>
         </is>
       </c>
       <c r="B861" t="inlineStr">
@@ -35836,12 +35836,12 @@
       </c>
       <c r="C861" t="inlineStr">
         <is>
-          <t>ingridevidot@gmail.com</t>
+          <t>pougary.davila@orange.fr</t>
         </is>
       </c>
       <c r="D861" t="inlineStr">
         <is>
-          <t>0692 19 28 11</t>
+          <t>0692 01 24 79</t>
         </is>
       </c>
       <c r="E861" t="inlineStr">
@@ -35868,7 +35868,7 @@
     <row r="862">
       <c r="A862" t="inlineStr">
         <is>
-          <t>Mélanz à nous</t>
+          <t>Mathias Maloya</t>
         </is>
       </c>
       <c r="B862" t="inlineStr">
@@ -35878,12 +35878,12 @@
       </c>
       <c r="C862" t="inlineStr">
         <is>
-          <t>melanzanou@gmail.com</t>
+          <t>ingridevidot@gmail.com</t>
         </is>
       </c>
       <c r="D862" t="inlineStr">
         <is>
-          <t>0692 51 21 27</t>
+          <t>0692 19 28 11</t>
         </is>
       </c>
       <c r="E862" t="inlineStr">
@@ -35910,7 +35910,7 @@
     <row r="863">
       <c r="A863" t="inlineStr">
         <is>
-          <t>ZOT Y PIN</t>
+          <t>Mélanz à nous</t>
         </is>
       </c>
       <c r="B863" t="inlineStr">
@@ -35920,10 +35920,14 @@
       </c>
       <c r="C863" t="inlineStr">
         <is>
-          <t>clfougeroux@gmail.com</t>
-        </is>
-      </c>
-      <c r="D863" t="inlineStr"/>
+          <t>melanzanou@gmail.com</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>0692 51 21 27</t>
+        </is>
+      </c>
       <c r="E863" t="inlineStr">
         <is>
           <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
@@ -35948,37 +35952,33 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>A. Dimitile Inter Génération</t>
+          <t>ZOT Y PIN</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
         <is>
-          <t>Entre-Deux</t>
+          <t>Trois-Bassins</t>
         </is>
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>adig.reunion974@gmail.com</t>
-        </is>
-      </c>
-      <c r="D864" t="inlineStr">
-        <is>
-          <t>0692 48 43 56</t>
-        </is>
-      </c>
+          <t>clfougeroux@gmail.com</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr"/>
       <c r="E864" t="inlineStr">
         <is>
-          <t>https://www.entredeux.re/sites/default/files/2023-06/Le%20GUIDE%20des%20associations%20ED-2023.pdf</t>
+          <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
         </is>
       </c>
       <c r="F864" t="inlineStr">
         <is>
-          <t>2023-06-14 (PDF Guide des associations 2023, publie sur entredeux.re le 14/06/2023)</t>
+          <t>2023-11-21 (PDF annuaire des associations de Trois Bassins, MAJ 21/11/2023, docs.trois-bassins.re; site actif 2026)</t>
         </is>
       </c>
       <c r="G864" t="inlineStr">
         <is>
-          <t>solidarite</t>
+          <t>loisirs_culture</t>
         </is>
       </c>
       <c r="H864" t="inlineStr">
@@ -35990,7 +35990,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>AKOZ Association Cultures Océanes Zazakely</t>
+          <t>A. Dimitile Inter Génération</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -36000,12 +36000,12 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>asso974.acoz@gmail.com</t>
+          <t>adig.reunion974@gmail.com</t>
         </is>
       </c>
       <c r="D865" t="inlineStr">
         <is>
-          <t>06 92 65 57 39</t>
+          <t>0692 48 43 56</t>
         </is>
       </c>
       <c r="E865" t="inlineStr">
@@ -36032,7 +36032,7 @@
     <row r="866">
       <c r="A866" t="inlineStr">
         <is>
-          <t>JADE Jeune Association pour le Développement Économique et Social</t>
+          <t>AKOZ Association Cultures Océanes Zazakely</t>
         </is>
       </c>
       <c r="B866" t="inlineStr">
@@ -36042,12 +36042,12 @@
       </c>
       <c r="C866" t="inlineStr">
         <is>
-          <t>techer.jade@gmail.com</t>
+          <t>asso974.acoz@gmail.com</t>
         </is>
       </c>
       <c r="D866" t="inlineStr">
         <is>
-          <t>0262 59 99 26</t>
+          <t>06 92 65 57 39</t>
         </is>
       </c>
       <c r="E866" t="inlineStr">
@@ -36074,7 +36074,7 @@
     <row r="867">
       <c r="A867" t="inlineStr">
         <is>
-          <t>Jeunesse Malgache de Demain</t>
+          <t>JADE Jeune Association pour le Développement Économique et Social</t>
         </is>
       </c>
       <c r="B867" t="inlineStr">
@@ -36084,12 +36084,12 @@
       </c>
       <c r="C867" t="inlineStr">
         <is>
-          <t>jcsertier@gmail.com</t>
+          <t>techer.jade@gmail.com</t>
         </is>
       </c>
       <c r="D867" t="inlineStr">
         <is>
-          <t>0692 87 74 32</t>
+          <t>0262 59 99 26</t>
         </is>
       </c>
       <c r="E867" t="inlineStr">
@@ -36116,7 +36116,7 @@
     <row r="868">
       <c r="A868" t="inlineStr">
         <is>
-          <t>Reunis Sourds LFPC</t>
+          <t>Jeunesse Malgache de Demain</t>
         </is>
       </c>
       <c r="B868" t="inlineStr">
@@ -36126,12 +36126,12 @@
       </c>
       <c r="C868" t="inlineStr">
         <is>
-          <t>reunisourdslfpc@gmail.com</t>
+          <t>jcsertier@gmail.com</t>
         </is>
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>0692 10 31 20</t>
+          <t>0692 87 74 32</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
@@ -36158,7 +36158,7 @@
     <row r="869">
       <c r="A869" t="inlineStr">
         <is>
-          <t>Échange Solidaire Foulpointe Entre-Deux</t>
+          <t>Reunis Sourds LFPC</t>
         </is>
       </c>
       <c r="B869" t="inlineStr">
@@ -36168,12 +36168,12 @@
       </c>
       <c r="C869" t="inlineStr">
         <is>
-          <t>rivierelucien1@gmail.com</t>
+          <t>reunisourdslfpc@gmail.com</t>
         </is>
       </c>
       <c r="D869" t="inlineStr">
         <is>
-          <t>0692 26 52 15</t>
+          <t>0692 10 31 20</t>
         </is>
       </c>
       <c r="E869" t="inlineStr">
@@ -36200,32 +36200,32 @@
     <row r="870">
       <c r="A870" t="inlineStr">
         <is>
-          <t>Alon Feminisme Reunion</t>
+          <t>Échange Solidaire Foulpointe Entre-Deux</t>
         </is>
       </c>
       <c r="B870" t="inlineStr">
         <is>
-          <t>L'Étang-Salé</t>
+          <t>Entre-Deux</t>
         </is>
       </c>
       <c r="C870" t="inlineStr">
         <is>
-          <t>alonfeminismereunion@gmail.com</t>
+          <t>rivierelucien1@gmail.com</t>
         </is>
       </c>
       <c r="D870" t="inlineStr">
         <is>
-          <t>0692.88.15.73</t>
+          <t>0692 26 52 15</t>
         </is>
       </c>
       <c r="E870" t="inlineStr">
         <is>
-          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=2</t>
+          <t>https://www.entredeux.re/sites/default/files/2023-06/Le%20GUIDE%20des%20associations%20ED-2023.pdf</t>
         </is>
       </c>
       <c r="F870" t="inlineStr">
         <is>
-          <t>2026 (annuaire des associations letangsale.fr; site actif: (c) 2026, actualité du 2026-07-07)</t>
+          <t>2023-06-14 (PDF Guide des associations 2023, publie sur entredeux.re le 14/06/2023)</t>
         </is>
       </c>
       <c r="G870" t="inlineStr">
@@ -36235,14 +36235,14 @@
       </c>
       <c r="H870" t="inlineStr">
         <is>
-          <t>site_actif_sans_date</t>
+          <t>date</t>
         </is>
       </c>
     </row>
     <row r="871">
       <c r="A871" t="inlineStr">
         <is>
-          <t>Association Paloma</t>
+          <t>Alon Feminisme Reunion</t>
         </is>
       </c>
       <c r="B871" t="inlineStr">
@@ -36252,17 +36252,17 @@
       </c>
       <c r="C871" t="inlineStr">
         <is>
-          <t>direction@paloma.re</t>
+          <t>alonfeminismereunion@gmail.com</t>
         </is>
       </c>
       <c r="D871" t="inlineStr">
         <is>
-          <t>0692.64.45.54</t>
+          <t>0692.88.15.73</t>
         </is>
       </c>
       <c r="E871" t="inlineStr">
         <is>
-          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=7</t>
+          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=2</t>
         </is>
       </c>
       <c r="F871" t="inlineStr">
@@ -36284,7 +36284,7 @@
     <row r="872">
       <c r="A872" t="inlineStr">
         <is>
-          <t>Bulles A Creer Et Cultiver Le Bonheur</t>
+          <t>Association Paloma</t>
         </is>
       </c>
       <c r="B872" t="inlineStr">
@@ -36294,17 +36294,17 @@
       </c>
       <c r="C872" t="inlineStr">
         <is>
-          <t>bullesacreerlebonheur@gmail.com</t>
+          <t>direction@paloma.re</t>
         </is>
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>0692.05.83.36</t>
+          <t>0692.64.45.54</t>
         </is>
       </c>
       <c r="E872" t="inlineStr">
         <is>
-          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=5</t>
+          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=7</t>
         </is>
       </c>
       <c r="F872" t="inlineStr">
@@ -36326,7 +36326,7 @@
     <row r="873">
       <c r="A873" t="inlineStr">
         <is>
-          <t>Ex Aequo</t>
+          <t>Bulles A Creer Et Cultiver Le Bonheur</t>
         </is>
       </c>
       <c r="B873" t="inlineStr">
@@ -36336,12 +36336,12 @@
       </c>
       <c r="C873" t="inlineStr">
         <is>
-          <t>exaequo.fh@gmail.com</t>
+          <t>bullesacreerlebonheur@gmail.com</t>
         </is>
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>0692.70.52.49</t>
+          <t>0692.05.83.36</t>
         </is>
       </c>
       <c r="E873" t="inlineStr">
@@ -36368,7 +36368,7 @@
     <row r="874">
       <c r="A874" t="inlineStr">
         <is>
-          <t>Les Victimes Silencieuses</t>
+          <t>Ex Aequo</t>
         </is>
       </c>
       <c r="B874" t="inlineStr">
@@ -36378,17 +36378,17 @@
       </c>
       <c r="C874" t="inlineStr">
         <is>
-          <t>victimes.silencieuses@gmail.com</t>
+          <t>exaequo.fh@gmail.com</t>
         </is>
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>0692.28.27.29</t>
+          <t>0692.70.52.49</t>
         </is>
       </c>
       <c r="E874" t="inlineStr">
         <is>
-          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=2</t>
+          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=5</t>
         </is>
       </c>
       <c r="F874" t="inlineStr">
@@ -36410,7 +36410,7 @@
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>Run Odyssea</t>
+          <t>Les Victimes Silencieuses</t>
         </is>
       </c>
       <c r="B875" t="inlineStr">
@@ -36420,17 +36420,17 @@
       </c>
       <c r="C875" t="inlineStr">
         <is>
-          <t>contact@run-odyssea.org</t>
+          <t>victimes.silencieuses@gmail.com</t>
         </is>
       </c>
       <c r="D875" t="inlineStr">
         <is>
-          <t>0693.39.78.05</t>
+          <t>0692.28.27.29</t>
         </is>
       </c>
       <c r="E875" t="inlineStr">
         <is>
-          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=5</t>
+          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=2</t>
         </is>
       </c>
       <c r="F875" t="inlineStr">
@@ -36452,7 +36452,7 @@
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>Saf Ocean Indien</t>
+          <t>Run Odyssea</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
@@ -36462,17 +36462,17 @@
       </c>
       <c r="C876" t="inlineStr">
         <is>
-          <t>actionsocial.safoi@gmail.com</t>
+          <t>contact@run-odyssea.org</t>
         </is>
       </c>
       <c r="D876" t="inlineStr">
         <is>
-          <t>0692.87.57.87</t>
+          <t>0693.39.78.05</t>
         </is>
       </c>
       <c r="E876" t="inlineStr">
         <is>
-          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations</t>
+          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations?site=5</t>
         </is>
       </c>
       <c r="F876" t="inlineStr">
@@ -36494,28 +36494,32 @@
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>ADACAM 974</t>
+          <t>Saf Ocean Indien</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>La Possession</t>
+          <t>L'Étang-Salé</t>
         </is>
       </c>
       <c r="C877" t="inlineStr">
         <is>
-          <t>adacam974@gmail.com</t>
-        </is>
-      </c>
-      <c r="D877" t="inlineStr"/>
+          <t>actionsocial.safoi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>0692.87.57.87</t>
+        </is>
+      </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199582</t>
+          <t>https://www.letangsale.fr/mes-acces-rapides/mes-liens-utiles/annuaire-des-associations</t>
         </is>
       </c>
       <c r="F877" t="inlineStr">
         <is>
-          <t>2026 (fiche annuaire des associations lapossession.re; site actif: Copyright 2026, actualités oct. 2026)</t>
+          <t>2026 (annuaire des associations letangsale.fr; site actif: (c) 2026, actualité du 2026-07-07)</t>
         </is>
       </c>
       <c r="G877" t="inlineStr">
@@ -36532,7 +36536,7 @@
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>AHTPAP LOUISE MICHELLE</t>
+          <t>ADACAM 974</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
@@ -36542,13 +36546,13 @@
       </c>
       <c r="C878" t="inlineStr">
         <is>
-          <t>ahtpap.louisemichelle@gmail.com</t>
+          <t>adacam974@gmail.com</t>
         </is>
       </c>
       <c r="D878" t="inlineStr"/>
       <c r="E878" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199600</t>
+          <t>https://www.lapossession.re/associations/199582</t>
         </is>
       </c>
       <c r="F878" t="inlineStr">
@@ -36570,7 +36574,7 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>ARPS ASSOCIATION REUNIONNAISE POUR LA PREVENTION DES RISQUES LIES A LA SEXUALITE</t>
+          <t>AHTPAP LOUISE MICHELLE</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
@@ -36580,13 +36584,13 @@
       </c>
       <c r="C879" t="inlineStr">
         <is>
-          <t>administration@arps-info.com</t>
+          <t>ahtpap.louisemichelle@gmail.com</t>
         </is>
       </c>
       <c r="D879" t="inlineStr"/>
       <c r="E879" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199545</t>
+          <t>https://www.lapossession.re/associations/199600</t>
         </is>
       </c>
       <c r="F879" t="inlineStr">
@@ -36608,7 +36612,7 @@
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>ASSOCIATION ALLONS DEOR</t>
+          <t>ARPS ASSOCIATION REUNIONNAISE POUR LA PREVENTION DES RISQUES LIES A LA SEXUALITE</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
@@ -36618,13 +36622,13 @@
       </c>
       <c r="C880" t="inlineStr">
         <is>
-          <t>allons.deor@orange.fr</t>
+          <t>administration@arps-info.com</t>
         </is>
       </c>
       <c r="D880" t="inlineStr"/>
       <c r="E880" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199585</t>
+          <t>https://www.lapossession.re/associations/199545</t>
         </is>
       </c>
       <c r="F880" t="inlineStr">
@@ -36646,7 +36650,7 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>ASSOCIATION DEPARTEMENTALE HANDICAP MOTEUR DE LA REUNION (ADHMR)</t>
+          <t>ASSOCIATION ALLONS DEOR</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
@@ -36656,13 +36660,13 @@
       </c>
       <c r="C881" t="inlineStr">
         <is>
-          <t>adhmr974@gmail.com</t>
+          <t>allons.deor@orange.fr</t>
         </is>
       </c>
       <c r="D881" t="inlineStr"/>
       <c r="E881" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199564</t>
+          <t>https://www.lapossession.re/associations/199585</t>
         </is>
       </c>
       <c r="F881" t="inlineStr">
@@ -36684,7 +36688,7 @@
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>ASSOCIATION DES DIALYSES ET GREFFES DE LA REUNION</t>
+          <t>ASSOCIATION DEPARTEMENTALE HANDICAP MOTEUR DE LA REUNION (ADHMR)</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
@@ -36694,13 +36698,13 @@
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>adgreunion@gmail.com</t>
+          <t>adhmr974@gmail.com</t>
         </is>
       </c>
       <c r="D882" t="inlineStr"/>
       <c r="E882" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199547</t>
+          <t>https://www.lapossession.re/associations/199564</t>
         </is>
       </c>
       <c r="F882" t="inlineStr">
@@ -36722,7 +36726,7 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>ASSOCIATION FEMMES SOLID'AIR</t>
+          <t>ASSOCIATION DES DIALYSES ET GREFFES DE LA REUNION</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
@@ -36732,13 +36736,13 @@
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>femmes-solid.air@orange.fr</t>
+          <t>adgreunion@gmail.com</t>
         </is>
       </c>
       <c r="D883" t="inlineStr"/>
       <c r="E883" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199592</t>
+          <t>https://www.lapossession.re/associations/199547</t>
         </is>
       </c>
       <c r="F883" t="inlineStr">
@@ -36760,7 +36764,7 @@
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>ASSOCIATION FREDERIC LEVAVASSEUR</t>
+          <t>ASSOCIATION FEMMES SOLID'AIR</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
@@ -36770,13 +36774,13 @@
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>dlachenaye@afl.re</t>
+          <t>femmes-solid.air@orange.fr</t>
         </is>
       </c>
       <c r="D884" t="inlineStr"/>
       <c r="E884" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199561</t>
+          <t>https://www.lapossession.re/associations/199592</t>
         </is>
       </c>
       <c r="F884" t="inlineStr">
@@ -36798,7 +36802,7 @@
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>ASSOCIATION LES AMIS DE L'ECOLE PRIMAIRE PUBLIQUE D'AMBAHITRARAHABA MADAGASCAR</t>
+          <t>ASSOCIATION FREDERIC LEVAVASSEUR</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
@@ -36808,13 +36812,13 @@
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>stratus.berly@wanadoo.fr</t>
+          <t>dlachenaye@afl.re</t>
         </is>
       </c>
       <c r="D885" t="inlineStr"/>
       <c r="E885" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200215</t>
+          <t>https://www.lapossession.re/associations/199561</t>
         </is>
       </c>
       <c r="F885" t="inlineStr">
@@ -36836,7 +36840,7 @@
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
-          <t>ASSOCIATION RESEAU OTE</t>
+          <t>ASSOCIATION LES AMIS DE L'ECOLE PRIMAIRE PUBLIQUE D'AMBAHITRARAHABA MADAGASCAR</t>
         </is>
       </c>
       <c r="B886" t="inlineStr">
@@ -36846,13 +36850,13 @@
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>reseau.ote@wanadoo.fr</t>
+          <t>stratus.berly@wanadoo.fr</t>
         </is>
       </c>
       <c r="D886" t="inlineStr"/>
       <c r="E886" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199598</t>
+          <t>https://www.lapossession.re/associations/200215</t>
         </is>
       </c>
       <c r="F886" t="inlineStr">
@@ -36874,7 +36878,7 @@
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>ASSOCIATION RESEAU VIF</t>
+          <t>ASSOCIATION RESEAU OTE</t>
         </is>
       </c>
       <c r="B887" t="inlineStr">
@@ -36884,13 +36888,13 @@
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>contact@reseauvif.com</t>
+          <t>reseau.ote@wanadoo.fr</t>
         </is>
       </c>
       <c r="D887" t="inlineStr"/>
       <c r="E887" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199588</t>
+          <t>https://www.lapossession.re/associations/199598</t>
         </is>
       </c>
       <c r="F887" t="inlineStr">
@@ -36912,7 +36916,7 @@
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>AU TOUR DES BOURGEONS</t>
+          <t>ASSOCIATION RESEAU VIF</t>
         </is>
       </c>
       <c r="B888" t="inlineStr">
@@ -36922,13 +36926,13 @@
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>autourdesbourgeons@gmail.com</t>
+          <t>contact@reseauvif.com</t>
         </is>
       </c>
       <c r="D888" t="inlineStr"/>
       <c r="E888" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200231</t>
+          <t>https://www.lapossession.re/associations/199588</t>
         </is>
       </c>
       <c r="F888" t="inlineStr">
@@ -36950,7 +36954,7 @@
     <row r="889">
       <c r="A889" t="inlineStr">
         <is>
-          <t>BELLLS BIEN ETRE, LES LOISIRS &amp; LA SANTÉ</t>
+          <t>AU TOUR DES BOURGEONS</t>
         </is>
       </c>
       <c r="B889" t="inlineStr">
@@ -36960,13 +36964,13 @@
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>mcalogine@yahoo.com</t>
+          <t>autourdesbourgeons@gmail.com</t>
         </is>
       </c>
       <c r="D889" t="inlineStr"/>
       <c r="E889" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199557</t>
+          <t>https://www.lapossession.re/associations/200231</t>
         </is>
       </c>
       <c r="F889" t="inlineStr">
@@ -36988,7 +36992,7 @@
     <row r="890">
       <c r="A890" t="inlineStr">
         <is>
-          <t>CLAIRE JOIE</t>
+          <t>BELLLS BIEN ETRE, LES LOISIRS &amp; LA SANTÉ</t>
         </is>
       </c>
       <c r="B890" t="inlineStr">
@@ -36998,13 +37002,13 @@
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>secretariat@clairejoie.re</t>
+          <t>mcalogine@yahoo.com</t>
         </is>
       </c>
       <c r="D890" t="inlineStr"/>
       <c r="E890" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199560</t>
+          <t>https://www.lapossession.re/associations/199557</t>
         </is>
       </c>
       <c r="F890" t="inlineStr">
@@ -37026,7 +37030,7 @@
     <row r="891">
       <c r="A891" t="inlineStr">
         <is>
-          <t>COMPAGNON DE JE</t>
+          <t>CLAIRE JOIE</t>
         </is>
       </c>
       <c r="B891" t="inlineStr">
@@ -37036,13 +37040,13 @@
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>c2j@ecomail.re</t>
+          <t>secretariat@clairejoie.re</t>
         </is>
       </c>
       <c r="D891" t="inlineStr"/>
       <c r="E891" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199558</t>
+          <t>https://www.lapossession.re/associations/199560</t>
         </is>
       </c>
       <c r="F891" t="inlineStr">
@@ -37064,7 +37068,7 @@
     <row r="892">
       <c r="A892" t="inlineStr">
         <is>
-          <t>COMPAGNONS BATISSEURS DE LA RÉUNION</t>
+          <t>COMPAGNON DE JE</t>
         </is>
       </c>
       <c r="B892" t="inlineStr">
@@ -37074,13 +37078,13 @@
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>s.andoche@compagnonsbatisseurs.eu</t>
+          <t>c2j@ecomail.re</t>
         </is>
       </c>
       <c r="D892" t="inlineStr"/>
       <c r="E892" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199584</t>
+          <t>https://www.lapossession.re/associations/199558</t>
         </is>
       </c>
       <c r="F892" t="inlineStr">
@@ -37102,7 +37106,7 @@
     <row r="893">
       <c r="A893" t="inlineStr">
         <is>
-          <t>COPÉRATION RÉGIONALE OCÉAN INDIEN DE SPORT ADAPTÉ</t>
+          <t>COMPAGNONS BATISSEURS DE LA RÉUNION</t>
         </is>
       </c>
       <c r="B893" t="inlineStr">
@@ -37112,13 +37116,13 @@
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>c.r974@wanadoo.fr</t>
+          <t>s.andoche@compagnonsbatisseurs.eu</t>
         </is>
       </c>
       <c r="D893" t="inlineStr"/>
       <c r="E893" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199565</t>
+          <t>https://www.lapossession.re/associations/199584</t>
         </is>
       </c>
       <c r="F893" t="inlineStr">
@@ -37140,7 +37144,7 @@
     <row r="894">
       <c r="A894" t="inlineStr">
         <is>
-          <t>CŒUR DE FEMME</t>
+          <t>COPÉRATION RÉGIONALE OCÉAN INDIEN DE SPORT ADAPTÉ</t>
         </is>
       </c>
       <c r="B894" t="inlineStr">
@@ -37150,13 +37154,13 @@
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>coeurdefemme974@gmail.com</t>
+          <t>c.r974@wanadoo.fr</t>
         </is>
       </c>
       <c r="D894" t="inlineStr"/>
       <c r="E894" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200232</t>
+          <t>https://www.lapossession.re/associations/199565</t>
         </is>
       </c>
       <c r="F894" t="inlineStr">
@@ -37178,7 +37182,7 @@
     <row r="895">
       <c r="A895" t="inlineStr">
         <is>
-          <t>DEPIST' OUEST</t>
+          <t>CŒUR DE FEMME</t>
         </is>
       </c>
       <c r="B895" t="inlineStr">
@@ -37188,13 +37192,13 @@
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>thore.e@ch-gmartin.fr</t>
+          <t>coeurdefemme974@gmail.com</t>
         </is>
       </c>
       <c r="D895" t="inlineStr"/>
       <c r="E895" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199548</t>
+          <t>https://www.lapossession.re/associations/200232</t>
         </is>
       </c>
       <c r="F895" t="inlineStr">
@@ -37216,7 +37220,7 @@
     <row r="896">
       <c r="A896" t="inlineStr">
         <is>
-          <t>ECOL'O DE VIE</t>
+          <t>DEPIST' OUEST</t>
         </is>
       </c>
       <c r="B896" t="inlineStr">
@@ -37226,13 +37230,13 @@
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>ecolodevie@gmail.com</t>
+          <t>thore.e@ch-gmartin.fr</t>
         </is>
       </c>
       <c r="D896" t="inlineStr"/>
       <c r="E896" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200227</t>
+          <t>https://www.lapossession.re/associations/199548</t>
         </is>
       </c>
       <c r="F896" t="inlineStr">
@@ -37254,7 +37258,7 @@
     <row r="897">
       <c r="A897" t="inlineStr">
         <is>
-          <t>ED DA LI ZIZ PA LI</t>
+          <t>ECOL'O DE VIE</t>
         </is>
       </c>
       <c r="B897" t="inlineStr">
@@ -37264,13 +37268,13 @@
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>eloisemani441@gmail.com</t>
+          <t>ecolodevie@gmail.com</t>
         </is>
       </c>
       <c r="D897" t="inlineStr"/>
       <c r="E897" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200236</t>
+          <t>https://www.lapossession.re/associations/200227</t>
         </is>
       </c>
       <c r="F897" t="inlineStr">
@@ -37292,7 +37296,7 @@
     <row r="898">
       <c r="A898" t="inlineStr">
         <is>
-          <t>FEMMES CONNECTÉES</t>
+          <t>ED DA LI ZIZ PA LI</t>
         </is>
       </c>
       <c r="B898" t="inlineStr">
@@ -37302,13 +37306,13 @@
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>contact.femmesconnectees@gmail.com</t>
+          <t>eloisemani441@gmail.com</t>
         </is>
       </c>
       <c r="D898" t="inlineStr"/>
       <c r="E898" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/341139</t>
+          <t>https://www.lapossession.re/associations/200236</t>
         </is>
       </c>
       <c r="F898" t="inlineStr">
@@ -37330,7 +37334,7 @@
     <row r="899">
       <c r="A899" t="inlineStr">
         <is>
-          <t>GARD LESPOIR</t>
+          <t>FEMMES CONNECTÉES</t>
         </is>
       </c>
       <c r="B899" t="inlineStr">
@@ -37340,13 +37344,13 @@
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>gardlespoir@hotmail.com</t>
+          <t>contact.femmesconnectees@gmail.com</t>
         </is>
       </c>
       <c r="D899" t="inlineStr"/>
       <c r="E899" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199595</t>
+          <t>https://www.lapossession.re/associations/341139</t>
         </is>
       </c>
       <c r="F899" t="inlineStr">
@@ -37368,7 +37372,7 @@
     <row r="900">
       <c r="A900" t="inlineStr">
         <is>
-          <t>GRAMOUNS LE EN LER</t>
+          <t>GARD LESPOIR</t>
         </is>
       </c>
       <c r="B900" t="inlineStr">
@@ -37378,13 +37382,13 @@
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>lesgramouns974@gmail.com</t>
+          <t>gardlespoir@hotmail.com</t>
         </is>
       </c>
       <c r="D900" t="inlineStr"/>
       <c r="E900" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199604</t>
+          <t>https://www.lapossession.re/associations/199595</t>
         </is>
       </c>
       <c r="F900" t="inlineStr">
@@ -37406,7 +37410,7 @@
     <row r="901">
       <c r="A901" t="inlineStr">
         <is>
-          <t>HANDI RESILIENCE SOLIDARITE</t>
+          <t>GRAMOUNS LE EN LER</t>
         </is>
       </c>
       <c r="B901" t="inlineStr">
@@ -37416,13 +37420,13 @@
       </c>
       <c r="C901" t="inlineStr">
         <is>
-          <t>handiresol974@gmail.com</t>
+          <t>lesgramouns974@gmail.com</t>
         </is>
       </c>
       <c r="D901" t="inlineStr"/>
       <c r="E901" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200239</t>
+          <t>https://www.lapossession.re/associations/199604</t>
         </is>
       </c>
       <c r="F901" t="inlineStr">
@@ -37444,7 +37448,7 @@
     <row r="902">
       <c r="A902" t="inlineStr">
         <is>
-          <t>KADDY SOLIDAIRE</t>
+          <t>HANDI RESILIENCE SOLIDARITE</t>
         </is>
       </c>
       <c r="B902" t="inlineStr">
@@ -37454,13 +37458,13 @@
       </c>
       <c r="C902" t="inlineStr">
         <is>
-          <t>kaddy242426@gmail.com</t>
+          <t>handiresol974@gmail.com</t>
         </is>
       </c>
       <c r="D902" t="inlineStr"/>
       <c r="E902" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200216</t>
+          <t>https://www.lapossession.re/associations/200239</t>
         </is>
       </c>
       <c r="F902" t="inlineStr">
@@ -37482,7 +37486,7 @@
     <row r="903">
       <c r="A903" t="inlineStr">
         <is>
-          <t>KER SOLIDAIRE</t>
+          <t>KADDY SOLIDAIRE</t>
         </is>
       </c>
       <c r="B903" t="inlineStr">
@@ -37492,13 +37496,13 @@
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>mariejeannejessica7@gmail.com</t>
+          <t>kaddy242426@gmail.com</t>
         </is>
       </c>
       <c r="D903" t="inlineStr"/>
       <c r="E903" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200226</t>
+          <t>https://www.lapossession.re/associations/200216</t>
         </is>
       </c>
       <c r="F903" t="inlineStr">
@@ -37520,7 +37524,7 @@
     <row r="904">
       <c r="A904" t="inlineStr">
         <is>
-          <t>KOUD POUS'</t>
+          <t>KER SOLIDAIRE</t>
         </is>
       </c>
       <c r="B904" t="inlineStr">
@@ -37530,13 +37534,13 @@
       </c>
       <c r="C904" t="inlineStr">
         <is>
-          <t>koudpous974@gmail.com</t>
+          <t>mariejeannejessica7@gmail.com</t>
         </is>
       </c>
       <c r="D904" t="inlineStr"/>
       <c r="E904" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200225</t>
+          <t>https://www.lapossession.re/associations/200226</t>
         </is>
       </c>
       <c r="F904" t="inlineStr">
@@ -37558,7 +37562,7 @@
     <row r="905">
       <c r="A905" t="inlineStr">
         <is>
-          <t>KOULER LO KER</t>
+          <t>KOUD POUS'</t>
         </is>
       </c>
       <c r="B905" t="inlineStr">
@@ -37568,13 +37572,13 @@
       </c>
       <c r="C905" t="inlineStr">
         <is>
-          <t>stephane@koulerloker.com</t>
+          <t>koudpous974@gmail.com</t>
         </is>
       </c>
       <c r="D905" t="inlineStr"/>
       <c r="E905" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199559</t>
+          <t>https://www.lapossession.re/associations/200225</t>
         </is>
       </c>
       <c r="F905" t="inlineStr">
@@ -37596,7 +37600,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>KOZ ANSAMB</t>
+          <t>KOULER LO KER</t>
         </is>
       </c>
       <c r="B906" t="inlineStr">
@@ -37606,13 +37610,13 @@
       </c>
       <c r="C906" t="inlineStr">
         <is>
-          <t>kozansamb974@gmail.com</t>
+          <t>stephane@koulerloker.com</t>
         </is>
       </c>
       <c r="D906" t="inlineStr"/>
       <c r="E906" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199602</t>
+          <t>https://www.lapossession.re/associations/199559</t>
         </is>
       </c>
       <c r="F906" t="inlineStr">
@@ -37634,7 +37638,7 @@
     <row r="907">
       <c r="A907" t="inlineStr">
         <is>
-          <t>L'ARBRE A GRANDIR</t>
+          <t>KOZ ANSAMB</t>
         </is>
       </c>
       <c r="B907" t="inlineStr">
@@ -37644,13 +37648,13 @@
       </c>
       <c r="C907" t="inlineStr">
         <is>
-          <t>larbreagrandir@gmail.com</t>
+          <t>kozansamb974@gmail.com</t>
         </is>
       </c>
       <c r="D907" t="inlineStr"/>
       <c r="E907" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199578</t>
+          <t>https://www.lapossession.re/associations/199602</t>
         </is>
       </c>
       <c r="F907" t="inlineStr">
@@ -37672,7 +37676,7 @@
     <row r="908">
       <c r="A908" t="inlineStr">
         <is>
-          <t>L'ESSENCE DU LIEN</t>
+          <t>L'ARBRE A GRANDIR</t>
         </is>
       </c>
       <c r="B908" t="inlineStr">
@@ -37682,13 +37686,13 @@
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>lessencedulien@gmail.com</t>
+          <t>larbreagrandir@gmail.com</t>
         </is>
       </c>
       <c r="D908" t="inlineStr"/>
       <c r="E908" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199572</t>
+          <t>https://www.lapossession.re/associations/199578</t>
         </is>
       </c>
       <c r="F908" t="inlineStr">
@@ -37710,7 +37714,7 @@
     <row r="909">
       <c r="A909" t="inlineStr">
         <is>
-          <t>LA CAZE DU VIVRE ENSEMBLE</t>
+          <t>L'ESSENCE DU LIEN</t>
         </is>
       </c>
       <c r="B909" t="inlineStr">
@@ -37720,13 +37724,13 @@
       </c>
       <c r="C909" t="inlineStr">
         <is>
-          <t>lacazeduvivreensemble@gmail.com</t>
+          <t>lessencedulien@gmail.com</t>
         </is>
       </c>
       <c r="D909" t="inlineStr"/>
       <c r="E909" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200234</t>
+          <t>https://www.lapossession.re/associations/199572</t>
         </is>
       </c>
       <c r="F909" t="inlineStr">
@@ -37748,7 +37752,7 @@
     <row r="910">
       <c r="A910" t="inlineStr">
         <is>
-          <t>LA KAZ JOIE DE VIVRE</t>
+          <t>LA CAZE DU VIVRE ENSEMBLE</t>
         </is>
       </c>
       <c r="B910" t="inlineStr">
@@ -37758,13 +37762,13 @@
       </c>
       <c r="C910" t="inlineStr">
         <is>
-          <t>contact@joiedevivre.re</t>
+          <t>lacazeduvivreensemble@gmail.com</t>
         </is>
       </c>
       <c r="D910" t="inlineStr"/>
       <c r="E910" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200233</t>
+          <t>https://www.lapossession.re/associations/200234</t>
         </is>
       </c>
       <c r="F910" t="inlineStr">
@@ -37786,7 +37790,7 @@
     <row r="911">
       <c r="A911" t="inlineStr">
         <is>
-          <t>LA RUE FAMILLE DE FRANCE 974</t>
+          <t>LA KAZ JOIE DE VIVRE</t>
         </is>
       </c>
       <c r="B911" t="inlineStr">
@@ -37796,13 +37800,13 @@
       </c>
       <c r="C911" t="inlineStr">
         <is>
-          <t>antoinearaye@gmail.com</t>
+          <t>contact@joiedevivre.re</t>
         </is>
       </c>
       <c r="D911" t="inlineStr"/>
       <c r="E911" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199573</t>
+          <t>https://www.lapossession.re/associations/200233</t>
         </is>
       </c>
       <c r="F911" t="inlineStr">
@@ -37824,7 +37828,7 @@
     <row r="912">
       <c r="A912" t="inlineStr">
         <is>
-          <t>LE COLLECTIF EPA</t>
+          <t>LA RUE FAMILLE DE FRANCE 974</t>
         </is>
       </c>
       <c r="B912" t="inlineStr">
@@ -37834,13 +37838,13 @@
       </c>
       <c r="C912" t="inlineStr">
         <is>
-          <t>lecollectifepa@gmail.com</t>
+          <t>antoinearaye@gmail.com</t>
         </is>
       </c>
       <c r="D912" t="inlineStr"/>
       <c r="E912" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199591</t>
+          <t>https://www.lapossession.re/associations/199573</t>
         </is>
       </c>
       <c r="F912" t="inlineStr">
@@ -37862,7 +37866,7 @@
     <row r="913">
       <c r="A913" t="inlineStr">
         <is>
-          <t>LES IRIS</t>
+          <t>LE COLLECTIF EPA</t>
         </is>
       </c>
       <c r="B913" t="inlineStr">
@@ -37872,13 +37876,13 @@
       </c>
       <c r="C913" t="inlineStr">
         <is>
-          <t>associationlesiris@gmail.com</t>
+          <t>lecollectifepa@gmail.com</t>
         </is>
       </c>
       <c r="D913" t="inlineStr"/>
       <c r="E913" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200223</t>
+          <t>https://www.lapossession.re/associations/199591</t>
         </is>
       </c>
       <c r="F913" t="inlineStr">
@@ -37900,7 +37904,7 @@
     <row r="914">
       <c r="A914" t="inlineStr">
         <is>
-          <t>LES MALTRAITENCES, MOI J'EN PARLE !</t>
+          <t>LES IRIS</t>
         </is>
       </c>
       <c r="B914" t="inlineStr">
@@ -37910,13 +37914,13 @@
       </c>
       <c r="C914" t="inlineStr">
         <is>
-          <t>nathalie@les-maltraitances-moijenparle.fr</t>
+          <t>associationlesiris@gmail.com</t>
         </is>
       </c>
       <c r="D914" t="inlineStr"/>
       <c r="E914" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199590</t>
+          <t>https://www.lapossession.re/associations/200223</t>
         </is>
       </c>
       <c r="F914" t="inlineStr">
@@ -37938,7 +37942,7 @@
     <row r="915">
       <c r="A915" t="inlineStr">
         <is>
-          <t>LUDOKADOK</t>
+          <t>LES MALTRAITENCES, MOI J'EN PARLE !</t>
         </is>
       </c>
       <c r="B915" t="inlineStr">
@@ -37948,13 +37952,13 @@
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>ludokadok.lapossession@gmail.com</t>
+          <t>nathalie@les-maltraitances-moijenparle.fr</t>
         </is>
       </c>
       <c r="D915" t="inlineStr"/>
       <c r="E915" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200207</t>
+          <t>https://www.lapossession.re/associations/199590</t>
         </is>
       </c>
       <c r="F915" t="inlineStr">
@@ -37976,7 +37980,7 @@
     <row r="916">
       <c r="A916" t="inlineStr">
         <is>
-          <t>LÉ ENKOR TEMPS</t>
+          <t>LUDOKADOK</t>
         </is>
       </c>
       <c r="B916" t="inlineStr">
@@ -37986,13 +37990,13 @@
       </c>
       <c r="C916" t="inlineStr">
         <is>
-          <t>bonjour@letsgo.re</t>
+          <t>ludokadok.lapossession@gmail.com</t>
         </is>
       </c>
       <c r="D916" t="inlineStr"/>
       <c r="E916" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199583</t>
+          <t>https://www.lapossession.re/associations/200207</t>
         </is>
       </c>
       <c r="F916" t="inlineStr">
@@ -38014,7 +38018,7 @@
     <row r="917">
       <c r="A917" t="inlineStr">
         <is>
-          <t>MAISON DU DIABETE</t>
+          <t>LÉ ENKOR TEMPS</t>
         </is>
       </c>
       <c r="B917" t="inlineStr">
@@ -38024,13 +38028,13 @@
       </c>
       <c r="C917" t="inlineStr">
         <is>
-          <t>maisondudiabete974.mdd@gmail.com</t>
+          <t>bonjour@letsgo.re</t>
         </is>
       </c>
       <c r="D917" t="inlineStr"/>
       <c r="E917" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199546</t>
+          <t>https://www.lapossession.re/associations/199583</t>
         </is>
       </c>
       <c r="F917" t="inlineStr">
@@ -38052,7 +38056,7 @@
     <row r="918">
       <c r="A918" t="inlineStr">
         <is>
-          <t>OFFRIR UNE GOUTTE D'EAU</t>
+          <t>MAISON DU DIABETE</t>
         </is>
       </c>
       <c r="B918" t="inlineStr">
@@ -38062,13 +38066,13 @@
       </c>
       <c r="C918" t="inlineStr">
         <is>
-          <t>offrirunegouttedeau@outlook.com</t>
+          <t>maisondudiabete974.mdd@gmail.com</t>
         </is>
       </c>
       <c r="D918" t="inlineStr"/>
       <c r="E918" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200217</t>
+          <t>https://www.lapossession.re/associations/199546</t>
         </is>
       </c>
       <c r="F918" t="inlineStr">
@@ -38090,7 +38094,7 @@
     <row r="919">
       <c r="A919" t="inlineStr">
         <is>
-          <t>PAIRE 2 CŒURS</t>
+          <t>OFFRIR UNE GOUTTE D'EAU</t>
         </is>
       </c>
       <c r="B919" t="inlineStr">
@@ -38100,13 +38104,13 @@
       </c>
       <c r="C919" t="inlineStr">
         <is>
-          <t>assopaire2coeurs@hotmail.fr</t>
+          <t>offrirunegouttedeau@outlook.com</t>
         </is>
       </c>
       <c r="D919" t="inlineStr"/>
       <c r="E919" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200224</t>
+          <t>https://www.lapossession.re/associations/200217</t>
         </is>
       </c>
       <c r="F919" t="inlineStr">
@@ -38128,7 +38132,7 @@
     <row r="920">
       <c r="A920" t="inlineStr">
         <is>
-          <t>REUNION MOELLE ESPOIR</t>
+          <t>PAIRE 2 CŒURS</t>
         </is>
       </c>
       <c r="B920" t="inlineStr">
@@ -38138,13 +38142,13 @@
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>reunionmoelleespoir@gmail.com</t>
+          <t>assopaire2coeurs@hotmail.fr</t>
         </is>
       </c>
       <c r="D920" t="inlineStr"/>
       <c r="E920" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199553</t>
+          <t>https://www.lapossession.re/associations/200224</t>
         </is>
       </c>
       <c r="F920" t="inlineStr">
@@ -38166,7 +38170,7 @@
     <row r="921">
       <c r="A921" t="inlineStr">
         <is>
-          <t>SAF OCEAN INDIEN (Syndrome Alcoolisation Fœtale)</t>
+          <t>REUNION MOELLE ESPOIR</t>
         </is>
       </c>
       <c r="B921" t="inlineStr">
@@ -38176,13 +38180,13 @@
       </c>
       <c r="C921" t="inlineStr">
         <is>
-          <t>contactsafoi@gmail.com</t>
+          <t>reunionmoelleespoir@gmail.com</t>
         </is>
       </c>
       <c r="D921" t="inlineStr"/>
       <c r="E921" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199551</t>
+          <t>https://www.lapossession.re/associations/199553</t>
         </is>
       </c>
       <c r="F921" t="inlineStr">
@@ -38204,7 +38208,7 @@
     <row r="922">
       <c r="A922" t="inlineStr">
         <is>
-          <t>SAKISOIGNE</t>
+          <t>SAF OCEAN INDIEN (Syndrome Alcoolisation Fœtale)</t>
         </is>
       </c>
       <c r="B922" t="inlineStr">
@@ -38214,17 +38218,13 @@
       </c>
       <c r="C922" t="inlineStr">
         <is>
-          <t>sakisoigne@gmail.com</t>
-        </is>
-      </c>
-      <c r="D922" t="inlineStr">
-        <is>
-          <t>0262 33 42 23</t>
-        </is>
-      </c>
+          <t>contactsafoi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr"/>
       <c r="E922" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200237</t>
+          <t>https://www.lapossession.re/associations/199551</t>
         </is>
       </c>
       <c r="F922" t="inlineStr">
@@ -38246,7 +38246,7 @@
     <row r="923">
       <c r="A923" t="inlineStr">
         <is>
-          <t>SAKURA</t>
+          <t>SAKISOIGNE</t>
         </is>
       </c>
       <c r="B923" t="inlineStr">
@@ -38256,13 +38256,17 @@
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>erick@sakura974.re</t>
-        </is>
-      </c>
-      <c r="D923" t="inlineStr"/>
+          <t>sakisoigne@gmail.com</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>0262 33 42 23</t>
+        </is>
+      </c>
       <c r="E923" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200241</t>
+          <t>https://www.lapossession.re/associations/200237</t>
         </is>
       </c>
       <c r="F923" t="inlineStr">
@@ -38284,7 +38288,7 @@
     <row r="924">
       <c r="A924" t="inlineStr">
         <is>
-          <t>SOLEY POUR TOUS</t>
+          <t>SAKURA</t>
         </is>
       </c>
       <c r="B924" t="inlineStr">
@@ -38294,13 +38298,13 @@
       </c>
       <c r="C924" t="inlineStr">
         <is>
-          <t>soleypourtous@gmail.com</t>
+          <t>erick@sakura974.re</t>
         </is>
       </c>
       <c r="D924" t="inlineStr"/>
       <c r="E924" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200238</t>
+          <t>https://www.lapossession.re/associations/200241</t>
         </is>
       </c>
       <c r="F924" t="inlineStr">
@@ -38322,7 +38326,7 @@
     <row r="925">
       <c r="A925" t="inlineStr">
         <is>
-          <t>SOS GRAMOUNES ISOLÉS</t>
+          <t>SOLEY POUR TOUS</t>
         </is>
       </c>
       <c r="B925" t="inlineStr">
@@ -38332,13 +38336,13 @@
       </c>
       <c r="C925" t="inlineStr">
         <is>
-          <t>louaiselpatrice@gmail.com</t>
+          <t>soleypourtous@gmail.com</t>
         </is>
       </c>
       <c r="D925" t="inlineStr"/>
       <c r="E925" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199601</t>
+          <t>https://www.lapossession.re/associations/200238</t>
         </is>
       </c>
       <c r="F925" t="inlineStr">
@@ -38360,7 +38364,7 @@
     <row r="926">
       <c r="A926" t="inlineStr">
         <is>
-          <t>SOS SOLITUDE</t>
+          <t>SOS GRAMOUNES ISOLÉS</t>
         </is>
       </c>
       <c r="B926" t="inlineStr">
@@ -38370,13 +38374,13 @@
       </c>
       <c r="C926" t="inlineStr">
         <is>
-          <t>sossol974@gmail.com</t>
+          <t>louaiselpatrice@gmail.com</t>
         </is>
       </c>
       <c r="D926" t="inlineStr"/>
       <c r="E926" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199597</t>
+          <t>https://www.lapossession.re/associations/199601</t>
         </is>
       </c>
       <c r="F926" t="inlineStr">
@@ -38398,7 +38402,7 @@
     <row r="927">
       <c r="A927" t="inlineStr">
         <is>
-          <t>SPECIAL OLYMPICS REUNION</t>
+          <t>SOS SOLITUDE</t>
         </is>
       </c>
       <c r="B927" t="inlineStr">
@@ -38408,13 +38412,13 @@
       </c>
       <c r="C927" t="inlineStr">
         <is>
-          <t>soreunionchair@gmail.com</t>
+          <t>sossol974@gmail.com</t>
         </is>
       </c>
       <c r="D927" t="inlineStr"/>
       <c r="E927" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200240</t>
+          <t>https://www.lapossession.re/associations/199597</t>
         </is>
       </c>
       <c r="F927" t="inlineStr">
@@ -38436,7 +38440,7 @@
     <row r="928">
       <c r="A928" t="inlineStr">
         <is>
-          <t>SYNERGIE FAMILIE</t>
+          <t>SPECIAL OLYMPICS REUNION</t>
         </is>
       </c>
       <c r="B928" t="inlineStr">
@@ -38446,13 +38450,13 @@
       </c>
       <c r="C928" t="inlineStr">
         <is>
-          <t>mathilde.roux@synergiefamily.com</t>
+          <t>soreunionchair@gmail.com</t>
         </is>
       </c>
       <c r="D928" t="inlineStr"/>
       <c r="E928" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199570</t>
+          <t>https://www.lapossession.re/associations/200240</t>
         </is>
       </c>
       <c r="F928" t="inlineStr">
@@ -38474,7 +38478,7 @@
     <row r="929">
       <c r="A929" t="inlineStr">
         <is>
-          <t>TU ES MON AUTRE</t>
+          <t>SYNERGIE FAMILIE</t>
         </is>
       </c>
       <c r="B929" t="inlineStr">
@@ -38484,13 +38488,13 @@
       </c>
       <c r="C929" t="inlineStr">
         <is>
-          <t>asso.tuesmonautre@gmail.com</t>
+          <t>mathilde.roux@synergiefamily.com</t>
         </is>
       </c>
       <c r="D929" t="inlineStr"/>
       <c r="E929" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200218</t>
+          <t>https://www.lapossession.re/associations/199570</t>
         </is>
       </c>
       <c r="F929" t="inlineStr">
@@ -38512,7 +38516,7 @@
     <row r="930">
       <c r="A930" t="inlineStr">
         <is>
-          <t>UN AVENIR POUR TOUS</t>
+          <t>TU ES MON AUTRE</t>
         </is>
       </c>
       <c r="B930" t="inlineStr">
@@ -38522,13 +38526,13 @@
       </c>
       <c r="C930" t="inlineStr">
         <is>
-          <t>mireille.chungchin@gmail.com</t>
+          <t>asso.tuesmonautre@gmail.com</t>
         </is>
       </c>
       <c r="D930" t="inlineStr"/>
       <c r="E930" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200229</t>
+          <t>https://www.lapossession.re/associations/200218</t>
         </is>
       </c>
       <c r="F930" t="inlineStr">
@@ -38550,7 +38554,7 @@
     <row r="931">
       <c r="A931" t="inlineStr">
         <is>
-          <t>UN CŒUR C'EST UN CŒUR</t>
+          <t>UN AVENIR POUR TOUS</t>
         </is>
       </c>
       <c r="B931" t="inlineStr">
@@ -38560,13 +38564,13 @@
       </c>
       <c r="C931" t="inlineStr">
         <is>
-          <t>fabrice@uncoeurcestuncoeur.re</t>
+          <t>mireille.chungchin@gmail.com</t>
         </is>
       </c>
       <c r="D931" t="inlineStr"/>
       <c r="E931" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200228</t>
+          <t>https://www.lapossession.re/associations/200229</t>
         </is>
       </c>
       <c r="F931" t="inlineStr">
@@ -38588,7 +38592,7 @@
     <row r="932">
       <c r="A932" t="inlineStr">
         <is>
-          <t>UN FRUIT DE LA PASSION</t>
+          <t>UN CŒUR C'EST UN CŒUR</t>
         </is>
       </c>
       <c r="B932" t="inlineStr">
@@ -38598,13 +38602,13 @@
       </c>
       <c r="C932" t="inlineStr">
         <is>
-          <t>unfruitdelapassion974@gmail.com</t>
+          <t>fabrice@uncoeurcestuncoeur.re</t>
         </is>
       </c>
       <c r="D932" t="inlineStr"/>
       <c r="E932" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/200230</t>
+          <t>https://www.lapossession.re/associations/200228</t>
         </is>
       </c>
       <c r="F932" t="inlineStr">
@@ -38626,7 +38630,7 @@
     <row r="933">
       <c r="A933" t="inlineStr">
         <is>
-          <t>VIVRE AVEC LE S.A.F</t>
+          <t>UN FRUIT DE LA PASSION</t>
         </is>
       </c>
       <c r="B933" t="inlineStr">
@@ -38636,13 +38640,13 @@
       </c>
       <c r="C933" t="inlineStr">
         <is>
-          <t>vivreaveclesaf.oi@gmail.com</t>
+          <t>unfruitdelapassion974@gmail.com</t>
         </is>
       </c>
       <c r="D933" t="inlineStr"/>
       <c r="E933" t="inlineStr">
         <is>
-          <t>https://www.lapossession.re/associations/199552</t>
+          <t>https://www.lapossession.re/associations/200230</t>
         </is>
       </c>
       <c r="F933" t="inlineStr">
@@ -38664,32 +38668,28 @@
     <row r="934">
       <c r="A934" t="inlineStr">
         <is>
-          <t>Association Liaison</t>
+          <t>VIVRE AVEC LE S.A.F</t>
         </is>
       </c>
       <c r="B934" t="inlineStr">
         <is>
-          <t>Le Port</t>
+          <t>La Possession</t>
         </is>
       </c>
       <c r="C934" t="inlineStr">
         <is>
-          <t>liaison.association@hotmail.fr</t>
-        </is>
-      </c>
-      <c r="D934" t="inlineStr">
-        <is>
-          <t>0262 43 16 15</t>
-        </is>
-      </c>
+          <t>vivreaveclesaf.oi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr"/>
       <c r="E934" t="inlineStr">
         <is>
-          <t>https://www.ville-port.re/annuaire-des-clubs-sportifs-2/</t>
+          <t>https://www.lapossession.re/associations/199552</t>
         </is>
       </c>
       <c r="F934" t="inlineStr">
         <is>
-          <t>2026 (annuaire des associations sportives portoises 2026/2027, page ville-port.re)</t>
+          <t>2026 (fiche annuaire des associations lapossession.re; site actif: Copyright 2026, actualités oct. 2026)</t>
         </is>
       </c>
       <c r="G934" t="inlineStr">
@@ -38699,14 +38699,14 @@
       </c>
       <c r="H934" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>site_actif_sans_date</t>
         </is>
       </c>
     </row>
     <row r="935">
       <c r="A935" t="inlineStr">
         <is>
-          <t>Association Prévention Éducation Recherche Formation REED</t>
+          <t>Association Liaison</t>
         </is>
       </c>
       <c r="B935" t="inlineStr">
@@ -38716,12 +38716,12 @@
       </c>
       <c r="C935" t="inlineStr">
         <is>
-          <t>sec.aperf974@gmail.com</t>
+          <t>liaison.association@hotmail.fr</t>
         </is>
       </c>
       <c r="D935" t="inlineStr">
         <is>
-          <t>0692 68 34 34</t>
+          <t>0262 43 16 15</t>
         </is>
       </c>
       <c r="E935" t="inlineStr">
@@ -38748,32 +38748,32 @@
     <row r="936">
       <c r="A936" t="inlineStr">
         <is>
-          <t>Refuge Ti Lou (protection animale)</t>
+          <t>Association Prévention Éducation Recherche Formation REED</t>
         </is>
       </c>
       <c r="B936" t="inlineStr">
         <is>
-          <t>Le Tampon</t>
+          <t>Le Port</t>
         </is>
       </c>
       <c r="C936" t="inlineStr">
         <is>
-          <t>contact@tilou.re</t>
+          <t>sec.aperf974@gmail.com</t>
         </is>
       </c>
       <c r="D936" t="inlineStr">
         <is>
-          <t>09 76 31 68 99</t>
+          <t>0692 68 34 34</t>
         </is>
       </c>
       <c r="E936" t="inlineStr">
         <is>
-          <t>https://letampon.fr/wp-content/uploads/2026/02/Tampon-magazine-68-mars-2026.pdf</t>
+          <t>https://www.ville-port.re/annuaire-des-clubs-sportifs-2/</t>
         </is>
       </c>
       <c r="F936" t="inlineStr">
         <is>
-          <t>2026-03 (PDF Tampon Magazine n°68, mars 2026)</t>
+          <t>2026 (annuaire des associations sportives portoises 2026/2027, page ville-port.re)</t>
         </is>
       </c>
       <c r="G936" t="inlineStr">
@@ -38790,32 +38790,32 @@
     <row r="937">
       <c r="A937" t="inlineStr">
         <is>
-          <t>Des Aidants et des Aidés 974 (AAA 974)</t>
+          <t>Refuge Ti Lou (protection animale)</t>
         </is>
       </c>
       <c r="B937" t="inlineStr">
         <is>
-          <t>Petite-Île</t>
+          <t>Le Tampon</t>
         </is>
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>associationaaa974@gmail.com</t>
+          <t>contact@tilou.re</t>
         </is>
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>0692 52 44 81</t>
+          <t>09 76 31 68 99</t>
         </is>
       </c>
       <c r="E937" t="inlineStr">
         <is>
-          <t>https://www.petite-ile.re/ma-ville/associations</t>
+          <t>https://letampon.fr/wp-content/uploads/2026/02/Tampon-magazine-68-mars-2026.pdf</t>
         </is>
       </c>
       <c r="F937" t="inlineStr">
         <is>
-          <t>2026 - annuaire en ligne de la mairie (pages ?page=0 a 9), non date par page ; site mairie actif (bulletins sanitaires jusqu'a sept. 2026, copyright 2026)</t>
+          <t>2026-03 (PDF Tampon Magazine n°68, mars 2026)</t>
         </is>
       </c>
       <c r="G937" t="inlineStr">
@@ -38825,14 +38825,14 @@
       </c>
       <c r="H937" t="inlineStr">
         <is>
-          <t>site_actif_sans_date</t>
+          <t>date</t>
         </is>
       </c>
     </row>
     <row r="938">
       <c r="A938" t="inlineStr">
         <is>
-          <t>Développement d'Actions Sociales et Environnementales (ADASE)</t>
+          <t>Des Aidants et des Aidés 974 (AAA 974)</t>
         </is>
       </c>
       <c r="B938" t="inlineStr">
@@ -38842,12 +38842,12 @@
       </c>
       <c r="C938" t="inlineStr">
         <is>
-          <t>danielbriandy@orange.fr</t>
+          <t>associationaaa974@gmail.com</t>
         </is>
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>0692 87 56 42 - 0692 87 72 88</t>
+          <t>0692 52 44 81</t>
         </is>
       </c>
       <c r="E938" t="inlineStr">
@@ -38874,7 +38874,7 @@
     <row r="939">
       <c r="A939" t="inlineStr">
         <is>
-          <t>Hilaros</t>
+          <t>Développement d'Actions Sociales et Environnementales (ADASE)</t>
         </is>
       </c>
       <c r="B939" t="inlineStr">
@@ -38884,12 +38884,12 @@
       </c>
       <c r="C939" t="inlineStr">
         <is>
-          <t>hilaros974@gmail.com</t>
+          <t>danielbriandy@orange.fr</t>
         </is>
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>0692 28 45 72</t>
+          <t>0692 87 56 42 - 0692 87 72 88</t>
         </is>
       </c>
       <c r="E939" t="inlineStr">
@@ -38916,7 +38916,7 @@
     <row r="940">
       <c r="A940" t="inlineStr">
         <is>
-          <t>Kalbass</t>
+          <t>Hilaros</t>
         </is>
       </c>
       <c r="B940" t="inlineStr">
@@ -38926,12 +38926,12 @@
       </c>
       <c r="C940" t="inlineStr">
         <is>
-          <t>kalbass97429@gmail.com</t>
+          <t>hilaros974@gmail.com</t>
         </is>
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>0693 50 02 35</t>
+          <t>0692 28 45 72</t>
         </is>
       </c>
       <c r="E940" t="inlineStr">
@@ -38958,7 +38958,7 @@
     <row r="941">
       <c r="A941" t="inlineStr">
         <is>
-          <t>Kréation pour l'Accompagnement Local des Ouvriers Unis (KALOU)</t>
+          <t>Kalbass</t>
         </is>
       </c>
       <c r="B941" t="inlineStr">
@@ -38968,12 +38968,12 @@
       </c>
       <c r="C941" t="inlineStr">
         <is>
-          <t>associationkalou@gmail.com</t>
+          <t>kalbass97429@gmail.com</t>
         </is>
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>0693 49 92 77</t>
+          <t>0693 50 02 35</t>
         </is>
       </c>
       <c r="E941" t="inlineStr">
@@ -39000,7 +39000,7 @@
     <row r="942">
       <c r="A942" t="inlineStr">
         <is>
-          <t>La Recyclerie du Sud</t>
+          <t>Kréation pour l'Accompagnement Local des Ouvriers Unis (KALOU)</t>
         </is>
       </c>
       <c r="B942" t="inlineStr">
@@ -39010,12 +39010,12 @@
       </c>
       <c r="C942" t="inlineStr">
         <is>
-          <t>pina.celine@yahoo.fr</t>
+          <t>associationkalou@gmail.com</t>
         </is>
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>0692 23 15 20</t>
+          <t>0693 49 92 77</t>
         </is>
       </c>
       <c r="E942" t="inlineStr">
@@ -39042,7 +39042,7 @@
     <row r="943">
       <c r="A943" t="inlineStr">
         <is>
-          <t>Les Samaritains</t>
+          <t>La Recyclerie du Sud</t>
         </is>
       </c>
       <c r="B943" t="inlineStr">
@@ -39052,12 +39052,12 @@
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>fredgigan97410@gmail.com</t>
+          <t>pina.celine@yahoo.fr</t>
         </is>
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>0693 94 62 55</t>
+          <t>0692 23 15 20</t>
         </is>
       </c>
       <c r="E943" t="inlineStr">
@@ -39084,7 +39084,7 @@
     <row r="944">
       <c r="A944" t="inlineStr">
         <is>
-          <t>Mouvement lé bon (MLB)</t>
+          <t>Les Samaritains</t>
         </is>
       </c>
       <c r="B944" t="inlineStr">
@@ -39094,12 +39094,12 @@
       </c>
       <c r="C944" t="inlineStr">
         <is>
-          <t>moutoussamvalfredine@gmail.com</t>
+          <t>fredgigan97410@gmail.com</t>
         </is>
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>0692 57 63 12</t>
+          <t>0693 94 62 55</t>
         </is>
       </c>
       <c r="E944" t="inlineStr">
@@ -39126,7 +39126,7 @@
     <row r="945">
       <c r="A945" t="inlineStr">
         <is>
-          <t>Médiation Familiale Sud Sauvage (AMF2S)</t>
+          <t>Mouvement lé bon (MLB)</t>
         </is>
       </c>
       <c r="B945" t="inlineStr">
@@ -39136,12 +39136,12 @@
       </c>
       <c r="C945" t="inlineStr">
         <is>
-          <t>asso.mf2s@gmail.com</t>
+          <t>moutoussamvalfredine@gmail.com</t>
         </is>
       </c>
       <c r="D945" t="inlineStr">
         <is>
-          <t>0262 30 68 50 - 0692 28 52 11</t>
+          <t>0692 57 63 12</t>
         </is>
       </c>
       <c r="E945" t="inlineStr">
@@ -39168,7 +39168,7 @@
     <row r="946">
       <c r="A946" t="inlineStr">
         <is>
-          <t>Un Geste, Un Sourire</t>
+          <t>Médiation Familiale Sud Sauvage (AMF2S)</t>
         </is>
       </c>
       <c r="B946" t="inlineStr">
@@ -39178,12 +39178,12 @@
       </c>
       <c r="C946" t="inlineStr">
         <is>
-          <t>ungesteunsourire@mailfence.com</t>
+          <t>asso.mf2s@gmail.com</t>
         </is>
       </c>
       <c r="D946" t="inlineStr">
         <is>
-          <t>0692 94 69 16</t>
+          <t>0262 30 68 50 - 0692 28 52 11</t>
         </is>
       </c>
       <c r="E946" t="inlineStr">
@@ -39210,7 +39210,7 @@
     <row r="947">
       <c r="A947" t="inlineStr">
         <is>
-          <t>Vivons Petite-Île</t>
+          <t>Un Geste, Un Sourire</t>
         </is>
       </c>
       <c r="B947" t="inlineStr">
@@ -39220,12 +39220,12 @@
       </c>
       <c r="C947" t="inlineStr">
         <is>
-          <t>gonthierfrederic8@gmail.com</t>
+          <t>ungesteunsourire@mailfence.com</t>
         </is>
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>0692 62 69 80</t>
+          <t>0692 94 69 16</t>
         </is>
       </c>
       <c r="E947" t="inlineStr">
@@ -39252,32 +39252,32 @@
     <row r="948">
       <c r="A948" t="inlineStr">
         <is>
-          <t>Association féminine de l'Est contre tristesse, tyrannie, traumatisme (AFECTTT)</t>
+          <t>Vivons Petite-Île</t>
         </is>
       </c>
       <c r="B948" t="inlineStr">
         <is>
-          <t>Saint-Benoît</t>
+          <t>Petite-Île</t>
         </is>
       </c>
       <c r="C948" t="inlineStr">
         <is>
-          <t>afecttt3@orange.fr</t>
+          <t>gonthierfrederic8@gmail.com</t>
         </is>
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>0692 61 76 59</t>
+          <t>0692 62 69 80</t>
         </is>
       </c>
       <c r="E948" t="inlineStr">
         <is>
-          <t>https://www.saint-benoit.re/page/475-associations-daction-sociale-humanitaire-entraide</t>
+          <t>https://www.petite-ile.re/ma-ville/associations</t>
         </is>
       </c>
       <c r="F948" t="inlineStr">
         <is>
-          <t>Page mairie non datée ; site mairie actif (actualités publiées 2026-10-19, rubrique Rouge Ruelle 2026), relevé 2026-10-20</t>
+          <t>2026 - annuaire en ligne de la mairie (pages ?page=0 a 9), non date par page ; site mairie actif (bulletins sanitaires jusqu'a sept. 2026, copyright 2026)</t>
         </is>
       </c>
       <c r="G948" t="inlineStr">
@@ -39294,7 +39294,7 @@
     <row r="949">
       <c r="A949" t="inlineStr">
         <is>
-          <t>Épi-Est</t>
+          <t>Association féminine de l'Est contre tristesse, tyrannie, traumatisme (AFECTTT)</t>
         </is>
       </c>
       <c r="B949" t="inlineStr">
@@ -39304,17 +39304,17 @@
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>epi.est@sfr.fr</t>
+          <t>afecttt3@orange.fr</t>
         </is>
       </c>
       <c r="D949" t="inlineStr">
         <is>
-          <t>0692 86 33 46</t>
+          <t>0692 61 76 59</t>
         </is>
       </c>
       <c r="E949" t="inlineStr">
         <is>
-          <t>https://www.saint-benoit.re/page/483-associations-de-linsertion</t>
+          <t>https://www.saint-benoit.re/page/475-associations-daction-sociale-humanitaire-entraide</t>
         </is>
       </c>
       <c r="F949" t="inlineStr">
@@ -39336,32 +39336,32 @@
     <row r="950">
       <c r="A950" t="inlineStr">
         <is>
-          <t>Psychez Toi</t>
+          <t>Épi-Est</t>
         </is>
       </c>
       <c r="B950" t="inlineStr">
         <is>
-          <t>Saint-Leu</t>
+          <t>Saint-Benoît</t>
         </is>
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>psycheztoi@gmail.com</t>
+          <t>epi.est@sfr.fr</t>
         </is>
       </c>
       <c r="D950" t="inlineStr">
         <is>
-          <t>06 93 92 04 23</t>
+          <t>0692 86 33 46</t>
         </is>
       </c>
       <c r="E950" t="inlineStr">
         <is>
-          <t>https://www.saintleu.re/fiche-association/psychez-toi</t>
+          <t>https://www.saint-benoit.re/page/483-associations-de-linsertion</t>
         </is>
       </c>
       <c r="F950" t="inlineStr">
         <is>
-          <t>2023-04-24 (fiche annuaire saintleu.re, dateModified; site actif 2026)</t>
+          <t>Page mairie non datée ; site mairie actif (actualités publiées 2026-10-19, rubrique Rouge Ruelle 2026), relevé 2026-10-20</t>
         </is>
       </c>
       <c r="G950" t="inlineStr">
@@ -39371,14 +39371,14 @@
       </c>
       <c r="H950" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>site_actif_sans_date</t>
         </is>
       </c>
     </row>
     <row r="951">
       <c r="A951" t="inlineStr">
         <is>
-          <t>Respirun</t>
+          <t>Psychez Toi</t>
         </is>
       </c>
       <c r="B951" t="inlineStr">
@@ -39388,18 +39388,22 @@
       </c>
       <c r="C951" t="inlineStr">
         <is>
-          <t>contact@respirun.org</t>
-        </is>
-      </c>
-      <c r="D951" t="inlineStr"/>
+          <t>psycheztoi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>06 93 92 04 23</t>
+        </is>
+      </c>
       <c r="E951" t="inlineStr">
         <is>
-          <t>https://www.saintleu.re/fiche-association/respirun</t>
+          <t>https://www.saintleu.re/fiche-association/psychez-toi</t>
         </is>
       </c>
       <c r="F951" t="inlineStr">
         <is>
-          <t>2023-08-04 (fiche annuaire saintleu.re, dateModified; site actif 2026)</t>
+          <t>2023-04-24 (fiche annuaire saintleu.re, dateModified; site actif 2026)</t>
         </is>
       </c>
       <c r="G951" t="inlineStr">
@@ -39416,7 +39420,7 @@
     <row r="952">
       <c r="A952" t="inlineStr">
         <is>
-          <t>Solidarité-Inter Génération</t>
+          <t>Respirun</t>
         </is>
       </c>
       <c r="B952" t="inlineStr">
@@ -39426,22 +39430,18 @@
       </c>
       <c r="C952" t="inlineStr">
         <is>
-          <t>daniel.faivre@yahoo.fr</t>
-        </is>
-      </c>
-      <c r="D952" t="inlineStr">
-        <is>
-          <t>0262 34 94 37 / 0692 23 92 49</t>
-        </is>
-      </c>
+          <t>contact@respirun.org</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr"/>
       <c r="E952" t="inlineStr">
         <is>
-          <t>https://www.saintleu.re/fiche-association/solidarite-inter-generation</t>
+          <t>https://www.saintleu.re/fiche-association/respirun</t>
         </is>
       </c>
       <c r="F952" t="inlineStr">
         <is>
-          <t>2022-04-21 (fiche annuaire saintleu.re, dateModified; site actif 2026)</t>
+          <t>2023-08-04 (fiche annuaire saintleu.re, dateModified; site actif 2026)</t>
         </is>
       </c>
       <c r="G952" t="inlineStr">
@@ -39458,32 +39458,32 @@
     <row r="953">
       <c r="A953" t="inlineStr">
         <is>
-          <t>Association Solidarité Sainte Thérèse</t>
+          <t>Solidarité-Inter Génération</t>
         </is>
       </c>
       <c r="B953" t="inlineStr">
         <is>
-          <t>Saint-Pierre</t>
+          <t>Saint-Leu</t>
         </is>
       </c>
       <c r="C953" t="inlineStr">
         <is>
-          <t>sainte.therese410@gmail.com</t>
+          <t>daniel.faivre@yahoo.fr</t>
         </is>
       </c>
       <c r="D953" t="inlineStr">
         <is>
-          <t>06 93 90 99 79 / 02 62 91 75 79</t>
+          <t>0262 34 94 37 / 0692 23 92 49</t>
         </is>
       </c>
       <c r="E953" t="inlineStr">
         <is>
-          <t>https://www.saintpierre.re/decouvrez-saint-pierre/le-cadre-de-vie/animations-vie-associative/repas-pour-les-demunis</t>
+          <t>https://www.saintleu.re/fiche-association/solidarite-inter-generation</t>
         </is>
       </c>
       <c r="F953" t="inlineStr">
         <is>
-          <t>2023-07-07 (actualite mairie, publie le 7 juillet 2023 ; association laique)</t>
+          <t>2022-04-21 (fiche annuaire saintleu.re, dateModified; site actif 2026)</t>
         </is>
       </c>
       <c r="G953" t="inlineStr">
@@ -39500,28 +39500,32 @@
     <row r="954">
       <c r="A954" t="inlineStr">
         <is>
-          <t>Association Réunionnaise pour le Développement de l'Insertion</t>
+          <t>Association Solidarité Sainte Thérèse</t>
         </is>
       </c>
       <c r="B954" t="inlineStr">
         <is>
-          <t>Trois-Bassins</t>
+          <t>Saint-Pierre</t>
         </is>
       </c>
       <c r="C954" t="inlineStr">
         <is>
-          <t>ardireunion@gmail.com</t>
-        </is>
-      </c>
-      <c r="D954" t="inlineStr"/>
+          <t>sainte.therese410@gmail.com</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>06 93 90 99 79 / 02 62 91 75 79</t>
+        </is>
+      </c>
       <c r="E954" t="inlineStr">
         <is>
-          <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
+          <t>https://www.saintpierre.re/decouvrez-saint-pierre/le-cadre-de-vie/animations-vie-associative/repas-pour-les-demunis</t>
         </is>
       </c>
       <c r="F954" t="inlineStr">
         <is>
-          <t>2023-11-21 (PDF annuaire des associations de Trois Bassins, MAJ 21/11/2023, docs.trois-bassins.re; site actif 2026)</t>
+          <t>2023-07-07 (actualite mairie, publie le 7 juillet 2023 ; association laique)</t>
         </is>
       </c>
       <c r="G954" t="inlineStr">
@@ -39538,47 +39542,85 @@
     <row r="955">
       <c r="A955" t="inlineStr">
         <is>
+          <t>Association Réunionnaise pour le Développement de l'Insertion</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Trois-Bassins</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>ardireunion@gmail.com</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr"/>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>2023-11-21 (PDF annuaire des associations de Trois Bassins, MAJ 21/11/2023, docs.trois-bassins.re; site actif 2026)</t>
+        </is>
+      </c>
+      <c r="G955" t="inlineStr">
+        <is>
+          <t>solidarite</t>
+        </is>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
           <t>Kfé parents</t>
         </is>
       </c>
-      <c r="B955" t="inlineStr">
+      <c r="B956" t="inlineStr">
         <is>
           <t>Trois-Bassins</t>
         </is>
       </c>
-      <c r="C955" t="inlineStr">
+      <c r="C956" t="inlineStr">
         <is>
           <t>monique.kfeparents@gmail.com</t>
         </is>
       </c>
-      <c r="D955" t="inlineStr">
+      <c r="D956" t="inlineStr">
         <is>
           <t>0262 82 42 73</t>
         </is>
       </c>
-      <c r="E955" t="inlineStr">
+      <c r="E956" t="inlineStr">
         <is>
           <t>https://docs.trois-bassins.re/associations/Liste-associations-3Bassins.pdf</t>
         </is>
       </c>
-      <c r="F955" t="inlineStr">
+      <c r="F956" t="inlineStr">
         <is>
           <t>2023-11-21 (PDF annuaire des associations de Trois Bassins, MAJ 21/11/2023, docs.trois-bassins.re; site actif 2026)</t>
         </is>
       </c>
-      <c r="G955" t="inlineStr">
+      <c r="G956" t="inlineStr">
         <is>
           <t>solidarite</t>
         </is>
       </c>
-      <c r="H955" t="inlineStr">
+      <c r="H956" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H955"/>
+  <autoFilter ref="A1:H956"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39853,7 +39895,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Pas d'annuaire ; page vie-associative en 404. Emails trouvés dans des arrêtés de manifestation/débit de boissons et le programme JEP publiés sur saintpierre.re (2024-2025). Écartés : Marmite Insolite (société commerciale), contacts d'agents (@saintpierre.re), Solidarité Sainte-Thérèse (déjà acquis). Quota Tavily 429 atteint ponctuellement ; les autres arrêtés (AJBS, Club Dominos Lé Margoz, Rugby Club, Run Power, Labelistic, Gaston Richardson) n'ont pas pu être lus en entier (extraction PDF échouée), emails non vérifiés donc non retenus.</t>
+          <t>802 PDF d'arrêtés de manifestations (2023-2026, tous scannés, OCR tesseract), 2173 autres PDF du site et 1487 pages analysés. Les arrêtés ne contiennent presque aucun email d'association : seuls VBSP, Saint-Pierre Handball Club (déjà acquis) et une SAS commerciale (Marmite Insolite, exclue) en ont un. Cibles sans email dans les arrêtés : Amicale des Jeunes Boulistes du Sud, Club Dominos Lé Margoz, Rugby Club Saint-Pierre et du Sud, Run Power Production, Labelistic (téléphone seul ou rien), Association Gaston Richardson (tél 06 92 87 85 73 seulement). Pages Maison Sport-Santé (OMS d'autres communes, CASEC, Ekilib) écartées : aucune date lisible sur la page. Le Vieux Domaine écarté (propriété privée, pas d'association nommée).</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">

</xml_diff>